<commit_message>
Resave product master template from Excel
</commit_message>
<xml_diff>
--- a/docs/templates/Nimbasia_Product_Master_Template.xlsx
+++ b/docs/templates/Nimbasia_Product_Master_Template.xlsx
@@ -1,42 +1,144 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nimbasia\docs\templates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_09F6971725BF89117423996D6074A9F580A597B3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Product Master" sheetId="1" r:id="rId1"/>
     <sheet name="Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
+  <si>
+    <t>Product Name</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Default Unit</t>
+  </si>
+  <si>
+    <t>HSN Code</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Opening Stock</t>
+  </si>
+  <si>
+    <t>Stearic Acid</t>
+  </si>
+  <si>
+    <t>RAW_MATERIAL</t>
+  </si>
+  <si>
+    <t>KG</t>
+  </si>
+  <si>
+    <t>38231900</t>
+  </si>
+  <si>
+    <t>Example row - delete before importing</t>
+  </si>
+  <si>
+    <t>Zinc Stearate Paper Bag</t>
+  </si>
+  <si>
+    <t>PACKING_MATERIAL</t>
+  </si>
+  <si>
+    <t>NOS</t>
+  </si>
+  <si>
+    <t>48194000</t>
+  </si>
+  <si>
+    <t>Zinc Stearate</t>
+  </si>
+  <si>
+    <t>FINISHED_GOODS</t>
+  </si>
+  <si>
+    <t>38249900</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>Must be unique. An existing name is UPDATED, a new one is created. Spelling must match the name already used in stock (e.g. 'Zinc Stearate', not 'ZINC STEARATE').</t>
+  </si>
+  <si>
+    <t>Recommended</t>
+  </si>
+  <si>
+    <t>One of: RAW_MATERIAL, PACKING_MATERIAL, FINISHED_GOODS. Decides which inventory screen the product's stock appears on. Also accepted: 'Raw Material', 'RM', 'Packing Material', 'Packing', 'Finished Goods', 'FG', 'Additive', 'Catalyst' (additives and catalysts count as raw material).</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>KG, MT, LTR, NOS etc. Used as the unit when the product has no stock history yet.</t>
+  </si>
+  <si>
+    <t>Tax classification code. Free text.</t>
+  </si>
+  <si>
+    <t>Free text notes.</t>
+  </si>
+  <si>
+    <t>Starting quantity. Applied on CREATE only - it is ignored when the product already exists, so re-importing cannot double-count stock. Leave blank for no opening stock.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>HOW TO IMPORT</t>
+  </si>
+  <si>
+    <t>Administration &gt; Product Master &gt; Import, then pick this file.</t>
+  </si>
+  <si>
+    <t>HEADER NAMES</t>
+  </si>
+  <si>
+    <t>Header spelling is flexible - 'Product'/'Item'/'Name' all map to Product Name, 'Type'/'Group' map to Category, 'Unit'/'UOM' map to Default Unit. Keep one header row.</t>
+  </si>
+  <si>
+    <t>DELETE EXAMPLES</t>
+  </si>
+  <si>
+    <t>Remove the three example rows before importing, or they will be created as real products.</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -66,13 +168,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -397,237 +507,240 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="40.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.796875" customWidth="1"/>
+    <col min="2" max="2" width="20.796875" customWidth="1"/>
+    <col min="3" max="4" width="14.796875" customWidth="1"/>
+    <col min="5" max="5" width="40.796875" customWidth="1"/>
+    <col min="6" max="6" width="14.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Product Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Category</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Default Unit</v>
-      </c>
-      <c r="D1" t="str">
-        <v>HSN Code</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Description</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Opening Stock</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Stearic Acid</v>
-      </c>
-      <c r="B2" t="str">
-        <v>RAW_MATERIAL</v>
-      </c>
-      <c r="C2" t="str">
-        <v>KG</v>
-      </c>
-      <c r="D2" t="str">
-        <v>38231900</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Example row - delete before importing</v>
+    <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
       </c>
       <c r="F2">
         <v>1000</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Zinc Stearate Paper Bag</v>
-      </c>
-      <c r="B3" t="str">
-        <v>PACKING_MATERIAL</v>
-      </c>
-      <c r="C3" t="str">
-        <v>NOS</v>
-      </c>
-      <c r="D3" t="str">
-        <v>48194000</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Example row - delete before importing</v>
+    <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
       </c>
       <c r="F3">
         <v>500</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Zinc Stearate</v>
-      </c>
-      <c r="B4" t="str">
-        <v>FINISHED_GOODS</v>
-      </c>
-      <c r="C4" t="str">
-        <v>KG</v>
-      </c>
-      <c r="D4" t="str">
-        <v>38249900</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Example row - delete before importing</v>
+    <row r="4" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError sqref="A1:F4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="110.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.796875" customWidth="1"/>
+    <col min="2" max="2" width="14.796875" customWidth="1"/>
+    <col min="3" max="3" width="110.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Field</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Required</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Product Name</v>
-      </c>
-      <c r="B2" t="str">
-        <v>YES</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Must be unique. An existing name is UPDATED, a new one is created. Spelling must match the name already used in stock (e.g. 'Zinc Stearate', not 'ZINC STEARATE').</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Category</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Recommended</v>
-      </c>
-      <c r="C3" t="str">
-        <v>One of: RAW_MATERIAL, PACKING_MATERIAL, FINISHED_GOODS. Decides which inventory screen the product's stock appears on. Also accepted: 'Raw Material', 'RM', 'Packing Material', 'Packing', 'Finished Goods', 'FG', 'Additive', 'Catalyst' (additives and catalysts count as raw material).</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Default Unit</v>
-      </c>
-      <c r="B4" t="str">
-        <v>No</v>
-      </c>
-      <c r="C4" t="str">
-        <v>KG, MT, LTR, NOS etc. Used as the unit when the product has no stock history yet.</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>HSN Code</v>
-      </c>
-      <c r="B5" t="str">
-        <v>No</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Tax classification code. Free text.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Description</v>
-      </c>
-      <c r="B6" t="str">
-        <v>No</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Free text notes.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Opening Stock</v>
-      </c>
-      <c r="B7" t="str">
-        <v>No</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Starting quantity. Applied on CREATE only - it is ignored when the product already exists, so re-importing cannot double-count stock. Leave blank for no opening stock.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v/>
-      </c>
-      <c r="B8" t="str">
-        <v/>
-      </c>
-      <c r="C8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>HOW TO IMPORT</v>
-      </c>
-      <c r="B9" t="str">
-        <v/>
-      </c>
-      <c r="C9" t="str">
-        <v>Administration &gt; Product Master &gt; Import, then pick this file.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>HEADER NAMES</v>
-      </c>
-      <c r="B10" t="str">
-        <v/>
-      </c>
-      <c r="C10" t="str">
-        <v>Header spelling is flexible - 'Product'/'Item'/'Name' all map to Product Name, 'Type'/'Group' map to Category, 'Unit'/'UOM' map to Default Unit. Keep one header row.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>DELETE EXAMPLES</v>
-      </c>
-      <c r="B11" t="str">
-        <v/>
-      </c>
-      <c r="C11" t="str">
-        <v>Remove the three example rows before importing, or they will be created as real products.</v>
+    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
+    <ignoredError sqref="A1:C11" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>